<commit_message>
docs: add m30 formal folder explanation and sheet row/column meanings
</commit_message>
<xml_diff>
--- a/04_结果/v4_正式版_m30/v4_每基金策略映射.xlsx
+++ b/04_结果/v4_正式版_m30/v4_每基金策略映射.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -443,6 +443,27 @@
       <c r="A3" t="inlineStr">
         <is>
           <t>每支基金最多 3-5 条策略；策略合并口径为同日取 |全历史 Average| 最大者。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>【行列含义】数据 Sheet：每行一条策略。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>列含义：基金名称（代码）、策略序号、触发条件、预测窗口（日）、全历史平均回报（%）、全历史交易数、全历史命中率、冻结期平均回报（%）、冻结期交易数、冻结期命中率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>策略命名规则：单条件如 SPY_up；双条件如 EEM_down_GDX_up；三条件如 FXY_up_up_down_GDX_QQQ；复合条件如 combo_QQQ_down__self_big_down；外部条件如 ext_vix_chg_ge5；自身条件如 self_3down。</t>
         </is>
       </c>
     </row>

</xml_diff>